<commit_message>
Publish strength guides and editorial trust signals
</commit_message>
<xml_diff>
--- a/seo-research/Kangoo_SEO_Keyword_Map_2026-06-11.xlsx
+++ b/seo-research/Kangoo_SEO_Keyword_Map_2026-06-11.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R6b629583390e4ec9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Map" sheetId="2" r:id="R45ef6dd772ee4021"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Roadmap" sheetId="3" r:id="R8237a225acf14d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cannibalisation" sheetId="4" r:id="R78a3a2ad542d43d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Files" sheetId="5" r:id="R2087c94a15c94c1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Re03b7d19a211479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keyword Map" sheetId="2" r:id="R2851842e2faa4f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Roadmap" sheetId="3" r:id="R966c9240cb2641a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cannibalisation" sheetId="4" r:id="R29c65bd8c1a64428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Files" sheetId="5" r:id="R06d88be871bb4cda"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -261,7 +261,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1296525f0bc5495a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc298ab409e584cbb"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -749,7 +749,7 @@
     <x:mergeCell ref="D3:H3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc519f4fbf8514f03"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76689cd0d7b743a3"/>
 </x:worksheet>
 </file>
 
@@ -34212,7 +34212,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raed130c0c25a471f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R111d10e72c804e05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34503,10 +34503,10 @@
         <x:v>/blog/3mg-nicotine-pouches/</x:v>
       </x:c>
       <x:c r="E14" s="4" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="F14" s="4" t="str">
-        <x:v>Weeks 2-4</x:v>
+        <x:v>Week 1</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -34523,10 +34523,10 @@
         <x:v>/blog/low-strength-nicotine-pouches/</x:v>
       </x:c>
       <x:c r="E15" s="4" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Implemented</x:v>
       </x:c>
       <x:c r="F15" s="4" t="str">
-        <x:v>Weeks 2-4</x:v>
+        <x:v>Week 1</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -34612,7 +34612,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R249a8bc535ff44cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c4bfc189dd84772"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34784,7 +34784,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bd5f7d11b7a48f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R858169a18ba14dbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>